<commit_message>
feat: fixed travel in quotation
</commit_message>
<xml_diff>
--- a/backend/storage/schema/quotation_template.xlsx
+++ b/backend/storage/schema/quotation_template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/longlh123/Languages/GitHub/IPSOS-FINANCE-PAYMENT/backend/storage/schema/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D91E1E71-337F-154D-87D4-BB59CE4C5716}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88C394AF-70E7-3243-9774-52639ED80C15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="6260" yWindow="3100" windowWidth="29040" windowHeight="17520" activeTab="1" xr2:uid="{C9138D76-07EC-41C4-8817-AFCBF30C50C2}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="541" uniqueCount="279">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="575" uniqueCount="293">
   <si>
     <t>field_name</t>
   </si>
@@ -187,9 +187,6 @@
     <t>Other</t>
   </si>
   <si>
-    <t>range</t>
-  </si>
-  <si>
     <t>default_value</t>
   </si>
   <si>
@@ -875,6 +872,51 @@
   </si>
   <si>
     <t>Yêu cầu về Quota</t>
+  </si>
+  <si>
+    <t>project_conditions</t>
+  </si>
+  <si>
+    <t>Điều kiện dự án</t>
+  </si>
+  <si>
+    <t>project_conditions_config</t>
+  </si>
+  <si>
+    <t>description</t>
+  </si>
+  <si>
+    <t>Đối tượng</t>
+  </si>
+  <si>
+    <t>travel_required</t>
+  </si>
+  <si>
+    <t>Yêu cầu Travel</t>
+  </si>
+  <si>
+    <t>travel_required_config</t>
+  </si>
+  <si>
+    <t>area</t>
+  </si>
+  <si>
+    <t>Area</t>
+  </si>
+  <si>
+    <t>excel:areas</t>
+  </si>
+  <si>
+    <t>areas</t>
+  </si>
+  <si>
+    <t>Urban</t>
+  </si>
+  <si>
+    <t>Rural</t>
+  </si>
+  <si>
+    <t>travel_comment</t>
   </si>
 </sst>
 </file>
@@ -1263,7 +1305,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6694FA44-4A7D-4629-A892-7DFDEEB80386}">
-  <dimension ref="A1:J23"/>
+  <dimension ref="A1:J25"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="24" bestFit="1" customWidth="1"/>
@@ -1289,27 +1331,27 @@
         <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>4</v>
       </c>
       <c r="H1" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="I1" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>55</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>56</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B2" t="s">
         <v>11</v>
@@ -1435,19 +1477,19 @@
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B8" t="s">
         <v>19</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D8">
         <v>1</v>
       </c>
       <c r="G8" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="H8">
         <v>12</v>
@@ -1461,7 +1503,7 @@
         <v>18</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D9">
         <v>1</v>
@@ -1475,7 +1517,7 @@
         <v>22</v>
       </c>
       <c r="B10" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>23</v>
@@ -1484,7 +1526,7 @@
         <v>1</v>
       </c>
       <c r="G10" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="H10">
         <v>12</v>
@@ -1492,19 +1534,19 @@
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
+        <v>161</v>
+      </c>
+      <c r="B11" t="s">
+        <v>160</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="D11">
+        <v>1</v>
+      </c>
+      <c r="F11" s="2" t="s">
         <v>162</v>
-      </c>
-      <c r="B11" t="s">
-        <v>161</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="D11">
-        <v>1</v>
-      </c>
-      <c r="F11" s="2" t="s">
-        <v>163</v>
       </c>
       <c r="H11">
         <v>12</v>
@@ -1512,10 +1554,10 @@
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
+        <v>77</v>
+      </c>
+      <c r="B12" t="s">
         <v>78</v>
-      </c>
-      <c r="B12" t="s">
-        <v>79</v>
       </c>
       <c r="C12" s="1" t="s">
         <v>28</v>
@@ -1524,7 +1566,7 @@
         <v>1</v>
       </c>
       <c r="F12" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H12">
         <v>12</v>
@@ -1532,19 +1574,19 @@
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
+        <v>61</v>
+      </c>
+      <c r="B13" t="s">
+        <v>60</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="D13">
+        <v>1</v>
+      </c>
+      <c r="F13" t="s">
         <v>62</v>
-      </c>
-      <c r="B13" t="s">
-        <v>61</v>
-      </c>
-      <c r="C13" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="D13">
-        <v>1</v>
-      </c>
-      <c r="F13" t="s">
-        <v>63</v>
       </c>
       <c r="H13">
         <v>12</v>
@@ -1552,19 +1594,16 @@
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>232</v>
+        <v>278</v>
       </c>
       <c r="B14" t="s">
-        <v>233</v>
+        <v>279</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="D14">
-        <v>1</v>
+        <v>82</v>
       </c>
       <c r="F14" t="s">
-        <v>232</v>
+        <v>280</v>
       </c>
       <c r="H14">
         <v>12</v>
@@ -1572,19 +1611,19 @@
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>112</v>
+        <v>231</v>
       </c>
       <c r="B15" t="s">
-        <v>111</v>
+        <v>232</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>28</v>
+        <v>82</v>
       </c>
       <c r="D15">
         <v>1</v>
       </c>
       <c r="F15" t="s">
-        <v>113</v>
+        <v>231</v>
       </c>
       <c r="H15">
         <v>12</v>
@@ -1592,19 +1631,19 @@
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
       <c r="B16" t="s">
-        <v>117</v>
+        <v>110</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>83</v>
+        <v>28</v>
       </c>
       <c r="D16">
         <v>1</v>
       </c>
       <c r="F16" t="s">
-        <v>118</v>
+        <v>112</v>
       </c>
       <c r="H16">
         <v>12</v>
@@ -1612,19 +1651,19 @@
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>131</v>
+        <v>115</v>
       </c>
       <c r="B17" t="s">
-        <v>132</v>
+        <v>116</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D17">
         <v>1</v>
       </c>
       <c r="F17" t="s">
-        <v>133</v>
+        <v>117</v>
       </c>
       <c r="H17">
         <v>12</v>
@@ -1632,19 +1671,19 @@
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>144</v>
+        <v>130</v>
       </c>
       <c r="B18" t="s">
-        <v>145</v>
+        <v>131</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D18">
         <v>1</v>
       </c>
       <c r="F18" t="s">
-        <v>146</v>
+        <v>132</v>
       </c>
       <c r="H18">
         <v>12</v>
@@ -1652,16 +1691,19 @@
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>205</v>
+        <v>143</v>
       </c>
       <c r="B19" t="s">
-        <v>204</v>
+        <v>144</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>57</v>
+        <v>82</v>
       </c>
       <c r="D19">
         <v>1</v>
+      </c>
+      <c r="F19" t="s">
+        <v>145</v>
       </c>
       <c r="H19">
         <v>12</v>
@@ -1669,19 +1711,16 @@
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="B20" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>23</v>
+        <v>56</v>
       </c>
       <c r="D20">
         <v>1</v>
-      </c>
-      <c r="G20" t="s">
-        <v>203</v>
       </c>
       <c r="H20">
         <v>12</v>
@@ -1689,19 +1728,19 @@
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>220</v>
+        <v>200</v>
       </c>
       <c r="B21" t="s">
-        <v>221</v>
+        <v>201</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>83</v>
+        <v>23</v>
       </c>
       <c r="D21">
         <v>1</v>
       </c>
-      <c r="F21" t="s">
-        <v>222</v>
+      <c r="G21" t="s">
+        <v>202</v>
       </c>
       <c r="H21">
         <v>12</v>
@@ -1709,19 +1748,19 @@
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>206</v>
+        <v>219</v>
       </c>
       <c r="B22" t="s">
-        <v>214</v>
+        <v>220</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>28</v>
+        <v>82</v>
       </c>
       <c r="D22">
         <v>1</v>
       </c>
       <c r="F22" t="s">
-        <v>207</v>
+        <v>221</v>
       </c>
       <c r="H22">
         <v>12</v>
@@ -1729,7 +1768,7 @@
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>212</v>
+        <v>205</v>
       </c>
       <c r="B23" t="s">
         <v>213</v>
@@ -1741,9 +1780,49 @@
         <v>1</v>
       </c>
       <c r="F23" t="s">
-        <v>215</v>
+        <v>206</v>
       </c>
       <c r="H23">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A24" t="s">
+        <v>211</v>
+      </c>
+      <c r="B24" t="s">
+        <v>212</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="D24">
+        <v>1</v>
+      </c>
+      <c r="F24" t="s">
+        <v>214</v>
+      </c>
+      <c r="H24">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A25" t="s">
+        <v>283</v>
+      </c>
+      <c r="B25" t="s">
+        <v>284</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="D25">
+        <v>1</v>
+      </c>
+      <c r="F25" t="s">
+        <v>285</v>
+      </c>
+      <c r="H25">
         <v>12</v>
       </c>
     </row>
@@ -1755,7 +1834,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F2B8FC54-75D4-4AC2-B92C-338AB72929A6}">
-  <dimension ref="A1:H55"/>
+  <dimension ref="A1:H59"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="29.83203125" bestFit="1" customWidth="1"/>
@@ -1784,114 +1863,114 @@
         <v>3</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>4</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B2" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E2">
         <v>1</v>
       </c>
       <c r="F2" s="1"/>
       <c r="G2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B3" t="s">
+        <v>193</v>
+      </c>
+      <c r="C3" t="s">
         <v>194</v>
       </c>
-      <c r="C3" t="s">
-        <v>195</v>
-      </c>
       <c r="D3" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E3">
         <v>1</v>
       </c>
       <c r="F3" s="1"/>
       <c r="G3" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="B4" t="s">
+        <v>164</v>
+      </c>
+      <c r="C4" t="s">
         <v>163</v>
       </c>
-      <c r="B4" t="s">
-        <v>165</v>
-      </c>
-      <c r="C4" t="s">
-        <v>164</v>
-      </c>
       <c r="D4" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E4">
         <v>1</v>
       </c>
       <c r="F4" s="1"/>
       <c r="G4" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B5" t="s">
+        <v>166</v>
+      </c>
+      <c r="C5" t="s">
         <v>167</v>
       </c>
-      <c r="C5" t="s">
-        <v>168</v>
-      </c>
       <c r="D5" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E5">
         <v>1</v>
       </c>
       <c r="F5" s="1"/>
       <c r="G5" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B6" t="s">
         <v>45</v>
@@ -1900,72 +1979,72 @@
         <v>20</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E6">
         <v>1</v>
       </c>
       <c r="F6" s="1"/>
       <c r="G6" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B7" t="s">
+        <v>187</v>
+      </c>
+      <c r="C7" t="s">
         <v>188</v>
       </c>
-      <c r="C7" t="s">
-        <v>189</v>
-      </c>
       <c r="D7" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E7">
         <v>1</v>
       </c>
       <c r="F7" s="1"/>
       <c r="H7" s="1" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
+        <v>79</v>
+      </c>
+      <c r="B8" t="s">
         <v>80</v>
-      </c>
-      <c r="B8" t="s">
-        <v>81</v>
       </c>
       <c r="C8" t="s">
         <v>41</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E8">
         <v>1</v>
       </c>
       <c r="G8" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B9" t="s">
         <v>25</v>
       </c>
       <c r="C9" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D9" s="1" t="s">
         <v>27</v>
@@ -1974,18 +2053,18 @@
         <v>1</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B10" t="s">
         <v>26</v>
       </c>
       <c r="C10" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D10" s="1" t="s">
         <v>27</v>
@@ -1994,182 +2073,181 @@
         <v>1</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B11" t="s">
-        <v>84</v>
+        <v>281</v>
       </c>
       <c r="C11" t="s">
-        <v>85</v>
+        <v>282</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>23</v>
+        <v>6</v>
       </c>
       <c r="E11">
         <v>1</v>
       </c>
-      <c r="G11" t="s">
-        <v>86</v>
-      </c>
       <c r="H11" s="1" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B12" t="s">
-        <v>90</v>
+        <v>83</v>
       </c>
       <c r="C12" t="s">
-        <v>91</v>
+        <v>84</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>49</v>
+        <v>23</v>
       </c>
       <c r="E12">
         <v>1</v>
       </c>
+      <c r="G12" t="s">
+        <v>85</v>
+      </c>
       <c r="H12" s="1" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B13" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="C13" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>60</v>
+        <v>6</v>
       </c>
       <c r="E13">
         <v>1</v>
       </c>
-      <c r="G13" t="s">
-        <v>94</v>
-      </c>
       <c r="H13" s="1" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>63</v>
+        <v>280</v>
       </c>
       <c r="B14" t="s">
-        <v>103</v>
+        <v>91</v>
       </c>
       <c r="C14" t="s">
-        <v>104</v>
+        <v>92</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="E14">
         <v>1</v>
       </c>
+      <c r="G14" t="s">
+        <v>93</v>
+      </c>
       <c r="H14" s="1" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>63</v>
+        <v>280</v>
       </c>
       <c r="B15" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C15" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E15">
         <v>1</v>
       </c>
       <c r="H15" s="1" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>63</v>
+        <v>280</v>
       </c>
       <c r="B16" t="s">
-        <v>248</v>
+        <v>100</v>
       </c>
       <c r="C16" t="s">
-        <v>276</v>
+        <v>101</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E16">
         <v>1</v>
       </c>
       <c r="H16" s="1" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>63</v>
+        <v>280</v>
       </c>
       <c r="B17" t="s">
-        <v>108</v>
+        <v>247</v>
       </c>
       <c r="C17" t="s">
-        <v>109</v>
+        <v>275</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E17">
         <v>1</v>
       </c>
       <c r="H17" s="1" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>232</v>
+        <v>280</v>
       </c>
       <c r="B18" t="s">
-        <v>180</v>
+        <v>107</v>
       </c>
       <c r="C18" t="s">
-        <v>183</v>
+        <v>108</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>27</v>
+        <v>56</v>
       </c>
       <c r="E18">
         <v>1</v>
       </c>
-      <c r="F18" s="1"/>
       <c r="H18" s="1" t="s">
         <v>192</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="B19" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="C19" t="s">
         <v>182</v>
@@ -2182,18 +2260,18 @@
       </c>
       <c r="F19" s="1"/>
       <c r="H19" s="1" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="B20" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="C20" t="s">
-        <v>186</v>
+        <v>181</v>
       </c>
       <c r="D20" s="1" t="s">
         <v>27</v>
@@ -2203,18 +2281,18 @@
       </c>
       <c r="F20" s="1"/>
       <c r="H20" s="1" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="B21" t="s">
+        <v>183</v>
+      </c>
+      <c r="C21" t="s">
         <v>185</v>
-      </c>
-      <c r="C21" t="s">
-        <v>187</v>
       </c>
       <c r="D21" s="1" t="s">
         <v>27</v>
@@ -2224,18 +2302,18 @@
       </c>
       <c r="F21" s="1"/>
       <c r="H21" s="1" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="B22" t="s">
-        <v>190</v>
+        <v>184</v>
       </c>
       <c r="C22" t="s">
-        <v>191</v>
+        <v>186</v>
       </c>
       <c r="D22" s="1" t="s">
         <v>27</v>
@@ -2245,63 +2323,60 @@
       </c>
       <c r="F22" s="1"/>
       <c r="H22" s="1" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="B23" t="s">
-        <v>234</v>
+        <v>189</v>
       </c>
       <c r="C23" t="s">
-        <v>235</v>
+        <v>190</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>57</v>
+        <v>27</v>
       </c>
       <c r="E23">
         <v>1</v>
       </c>
       <c r="F23" s="1"/>
       <c r="H23" s="1" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="B24" t="s">
-        <v>255</v>
+        <v>233</v>
       </c>
       <c r="C24" t="s">
-        <v>256</v>
+        <v>234</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>23</v>
+        <v>56</v>
       </c>
       <c r="E24">
         <v>1</v>
       </c>
       <c r="F24" s="1"/>
-      <c r="G24" t="s">
-        <v>51</v>
-      </c>
       <c r="H24" s="1" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="B25" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="C25" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="D25" s="1" t="s">
         <v>23</v>
@@ -2311,177 +2386,177 @@
       </c>
       <c r="F25" s="1"/>
       <c r="G25" t="s">
-        <v>259</v>
+        <v>50</v>
       </c>
       <c r="H25" s="1" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="B26" t="s">
-        <v>236</v>
+        <v>256</v>
       </c>
       <c r="C26" t="s">
-        <v>241</v>
+        <v>257</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>60</v>
+        <v>23</v>
       </c>
       <c r="E26">
         <v>1</v>
       </c>
       <c r="F26" s="1"/>
       <c r="G26" t="s">
-        <v>237</v>
+        <v>258</v>
       </c>
       <c r="H26" s="1" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="B27" t="s">
+        <v>235</v>
+      </c>
+      <c r="C27" t="s">
         <v>240</v>
       </c>
-      <c r="C27" t="s">
-        <v>242</v>
-      </c>
       <c r="D27" s="1" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="E27">
         <v>1</v>
       </c>
       <c r="F27" s="1"/>
+      <c r="G27" t="s">
+        <v>236</v>
+      </c>
       <c r="H27" s="1" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="B28" t="s">
-        <v>243</v>
+        <v>239</v>
       </c>
       <c r="C28" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E28">
         <v>1</v>
       </c>
       <c r="F28" s="1"/>
       <c r="H28" s="1" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="B29" t="s">
-        <v>254</v>
+        <v>242</v>
       </c>
       <c r="C29" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>23</v>
+        <v>56</v>
       </c>
       <c r="E29">
         <v>1</v>
       </c>
       <c r="F29" s="1"/>
-      <c r="G29" t="s">
-        <v>51</v>
-      </c>
       <c r="H29" s="1" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="B30" t="s">
-        <v>247</v>
+        <v>253</v>
       </c>
       <c r="C30" t="s">
         <v>245</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>57</v>
+        <v>23</v>
       </c>
       <c r="E30">
         <v>1</v>
       </c>
       <c r="F30" s="1"/>
+      <c r="G30" t="s">
+        <v>50</v>
+      </c>
       <c r="H30" s="1" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="B31" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="C31" t="s">
-        <v>249</v>
+        <v>244</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E31">
         <v>1</v>
       </c>
       <c r="F31" s="1"/>
       <c r="H31" s="1" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="B32" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="C32" t="s">
-        <v>252</v>
+        <v>248</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>23</v>
+        <v>56</v>
       </c>
       <c r="E32">
         <v>1</v>
       </c>
       <c r="F32" s="1"/>
-      <c r="G32" t="s">
-        <v>51</v>
-      </c>
       <c r="H32" s="1" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="B33" t="s">
+        <v>249</v>
+      </c>
+      <c r="C33" t="s">
         <v>251</v>
-      </c>
-      <c r="C33" t="s">
-        <v>253</v>
       </c>
       <c r="D33" s="1" t="s">
         <v>23</v>
@@ -2491,259 +2566,260 @@
       </c>
       <c r="F33" s="1"/>
       <c r="G33" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="H33" s="1" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>113</v>
+        <v>231</v>
       </c>
       <c r="B34" t="s">
-        <v>110</v>
+        <v>250</v>
       </c>
       <c r="C34" t="s">
-        <v>115</v>
+        <v>252</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>60</v>
+        <v>23</v>
       </c>
       <c r="E34">
         <v>1</v>
       </c>
+      <c r="F34" s="1"/>
       <c r="G34" t="s">
-        <v>114</v>
+        <v>50</v>
       </c>
       <c r="H34" s="1" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
+        <v>112</v>
+      </c>
+      <c r="B35" t="s">
+        <v>109</v>
+      </c>
+      <c r="C35" t="s">
+        <v>114</v>
+      </c>
+      <c r="D35" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="E35">
+        <v>1</v>
+      </c>
+      <c r="G35" t="s">
         <v>113</v>
       </c>
-      <c r="B35" t="s">
-        <v>227</v>
-      </c>
-      <c r="C35" t="s">
-        <v>229</v>
-      </c>
-      <c r="D35" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="E35">
-        <v>1</v>
-      </c>
-      <c r="F35">
-        <v>0</v>
-      </c>
       <c r="H35" s="1" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B36" t="s">
+        <v>226</v>
+      </c>
+      <c r="C36" t="s">
         <v>228</v>
-      </c>
-      <c r="C36" t="s">
-        <v>230</v>
       </c>
       <c r="D36" s="1" t="s">
         <v>27</v>
       </c>
       <c r="E36">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F36">
         <v>0</v>
       </c>
       <c r="H36" s="1" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>118</v>
+        <v>112</v>
       </c>
       <c r="B37" t="s">
-        <v>135</v>
+        <v>227</v>
       </c>
       <c r="C37" t="s">
-        <v>119</v>
+        <v>229</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>60</v>
+        <v>27</v>
       </c>
       <c r="E37">
-        <v>1</v>
-      </c>
-      <c r="G37" t="s">
-        <v>120</v>
+        <v>0</v>
+      </c>
+      <c r="F37">
+        <v>0</v>
       </c>
       <c r="H37" s="1" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
+        <v>117</v>
+      </c>
+      <c r="B38" t="s">
+        <v>134</v>
+      </c>
+      <c r="C38" t="s">
         <v>118</v>
       </c>
-      <c r="B38" t="s">
-        <v>136</v>
-      </c>
-      <c r="C38" t="s">
-        <v>126</v>
-      </c>
       <c r="D38" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E38">
         <v>1</v>
       </c>
       <c r="G38" t="s">
-        <v>127</v>
+        <v>119</v>
       </c>
       <c r="H38" s="1" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B39" t="s">
-        <v>277</v>
+        <v>135</v>
       </c>
       <c r="C39" t="s">
-        <v>278</v>
+        <v>125</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="E39">
         <v>1</v>
       </c>
+      <c r="G39" t="s">
+        <v>126</v>
+      </c>
       <c r="H39" s="1" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>133</v>
+        <v>117</v>
       </c>
       <c r="B40" t="s">
-        <v>141</v>
+        <v>276</v>
       </c>
       <c r="C40" t="s">
-        <v>134</v>
+        <v>277</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E40">
         <v>1</v>
       </c>
       <c r="H40" s="1" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
+        <v>132</v>
+      </c>
+      <c r="B41" t="s">
+        <v>140</v>
+      </c>
+      <c r="C41" t="s">
         <v>133</v>
       </c>
-      <c r="B41" t="s">
-        <v>137</v>
-      </c>
-      <c r="C41" t="s">
-        <v>138</v>
-      </c>
       <c r="D41" s="1" t="s">
-        <v>27</v>
+        <v>56</v>
       </c>
       <c r="E41">
         <v>1</v>
       </c>
       <c r="H41" s="1" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B42" t="s">
-        <v>142</v>
+        <v>136</v>
       </c>
       <c r="C42" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>57</v>
+        <v>27</v>
       </c>
       <c r="E42">
         <v>1</v>
       </c>
       <c r="H42" s="1" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B43" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="C43" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="D43" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E43">
         <v>1</v>
       </c>
       <c r="H43" s="1" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>146</v>
+        <v>132</v>
       </c>
       <c r="B44" t="s">
-        <v>147</v>
+        <v>142</v>
       </c>
       <c r="C44" t="s">
-        <v>149</v>
+        <v>139</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>23</v>
+        <v>56</v>
       </c>
       <c r="E44">
         <v>1</v>
       </c>
-      <c r="G44" t="s">
-        <v>51</v>
-      </c>
       <c r="H44" s="1" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
+        <v>145</v>
+      </c>
+      <c r="B45" t="s">
         <v>146</v>
       </c>
-      <c r="B45" t="s">
+      <c r="C45" t="s">
         <v>148</v>
-      </c>
-      <c r="C45" t="s">
-        <v>150</v>
       </c>
       <c r="D45" s="1" t="s">
         <v>23</v>
@@ -2752,219 +2828,308 @@
         <v>1</v>
       </c>
       <c r="G45" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="H45" s="1" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B46" t="s">
-        <v>160</v>
+        <v>147</v>
       </c>
       <c r="C46" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="D46" s="1" t="s">
-        <v>60</v>
+        <v>23</v>
       </c>
       <c r="E46">
         <v>1</v>
       </c>
       <c r="G46" t="s">
-        <v>154</v>
+        <v>50</v>
       </c>
       <c r="H46" s="1" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B47" t="s">
-        <v>152</v>
+        <v>159</v>
       </c>
       <c r="C47" t="s">
+        <v>150</v>
+      </c>
+      <c r="D47" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="E47">
+        <v>1</v>
+      </c>
+      <c r="G47" t="s">
         <v>153</v>
       </c>
-      <c r="D47" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="E47">
-        <v>1</v>
-      </c>
       <c r="H47" s="1" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
-        <v>222</v>
+        <v>145</v>
       </c>
       <c r="B48" t="s">
-        <v>223</v>
+        <v>151</v>
       </c>
       <c r="C48" t="s">
-        <v>224</v>
+        <v>152</v>
       </c>
       <c r="D48" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E48">
         <v>1</v>
       </c>
       <c r="H48" s="1" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
+        <v>221</v>
+      </c>
+      <c r="B49" t="s">
         <v>222</v>
       </c>
-      <c r="B49" t="s">
-        <v>225</v>
-      </c>
       <c r="C49" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D49" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E49">
         <v>1</v>
       </c>
       <c r="H49" s="1" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="50" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
-        <v>207</v>
+        <v>221</v>
       </c>
       <c r="B50" t="s">
-        <v>209</v>
+        <v>224</v>
       </c>
       <c r="C50" t="s">
-        <v>210</v>
+        <v>225</v>
       </c>
       <c r="D50" s="1" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="E50">
         <v>1</v>
       </c>
-      <c r="G50" t="s">
-        <v>114</v>
-      </c>
       <c r="H50" s="1" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="B51" t="s">
         <v>208</v>
       </c>
       <c r="C51" t="s">
-        <v>219</v>
+        <v>209</v>
       </c>
       <c r="D51" s="1" t="s">
-        <v>27</v>
+        <v>59</v>
       </c>
       <c r="E51">
         <v>1</v>
       </c>
+      <c r="G51" t="s">
+        <v>113</v>
+      </c>
       <c r="H51" s="1" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="52" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
+        <v>206</v>
+      </c>
+      <c r="B52" t="s">
         <v>207</v>
       </c>
-      <c r="B52" t="s">
-        <v>211</v>
-      </c>
       <c r="C52" t="s">
-        <v>189</v>
+        <v>218</v>
       </c>
       <c r="D52" s="1" t="s">
-        <v>6</v>
+        <v>27</v>
       </c>
       <c r="E52">
         <v>1</v>
       </c>
       <c r="H52" s="1" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="53" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
-        <v>215</v>
+        <v>206</v>
       </c>
       <c r="B53" t="s">
-        <v>217</v>
+        <v>210</v>
       </c>
       <c r="C53" t="s">
-        <v>210</v>
+        <v>188</v>
       </c>
       <c r="D53" s="1" t="s">
-        <v>60</v>
+        <v>6</v>
       </c>
       <c r="E53">
         <v>1</v>
       </c>
-      <c r="G53" t="s">
-        <v>114</v>
-      </c>
       <c r="H53" s="1" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="54" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="B54" t="s">
         <v>216</v>
       </c>
       <c r="C54" t="s">
-        <v>219</v>
+        <v>209</v>
       </c>
       <c r="D54" s="1" t="s">
-        <v>27</v>
+        <v>59</v>
       </c>
       <c r="E54">
         <v>1</v>
       </c>
+      <c r="G54" t="s">
+        <v>113</v>
+      </c>
       <c r="H54" s="1" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="55" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
+        <v>214</v>
+      </c>
+      <c r="B55" t="s">
         <v>215</v>
       </c>
-      <c r="B55" t="s">
+      <c r="C55" t="s">
         <v>218</v>
       </c>
-      <c r="C55" t="s">
-        <v>189</v>
-      </c>
       <c r="D55" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="E55">
+        <v>1</v>
+      </c>
+      <c r="H55" s="1" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="56" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A56" t="s">
+        <v>214</v>
+      </c>
+      <c r="B56" t="s">
+        <v>217</v>
+      </c>
+      <c r="C56" t="s">
+        <v>188</v>
+      </c>
+      <c r="D56" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="E55">
-        <v>1</v>
-      </c>
-      <c r="H55" s="1" t="s">
-        <v>193</v>
+      <c r="E56">
+        <v>1</v>
+      </c>
+      <c r="H56" s="1" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="57" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A57" t="s">
+        <v>285</v>
+      </c>
+      <c r="B57" t="s">
+        <v>109</v>
+      </c>
+      <c r="C57" t="s">
+        <v>114</v>
+      </c>
+      <c r="D57" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="E57">
+        <v>1</v>
+      </c>
+      <c r="G57" t="s">
+        <v>113</v>
+      </c>
+      <c r="H57" s="1" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="58" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A58" t="s">
+        <v>285</v>
+      </c>
+      <c r="B58" t="s">
+        <v>286</v>
+      </c>
+      <c r="C58" t="s">
+        <v>287</v>
+      </c>
+      <c r="D58" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="E58">
+        <v>1</v>
+      </c>
+      <c r="G58" t="s">
+        <v>288</v>
+      </c>
+      <c r="H58" s="1" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="59" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A59" t="s">
+        <v>285</v>
+      </c>
+      <c r="B59" t="s">
+        <v>292</v>
+      </c>
+      <c r="C59" t="s">
+        <v>188</v>
+      </c>
+      <c r="D59" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E59">
+        <v>1</v>
+      </c>
+      <c r="H59" s="1" t="s">
+        <v>192</v>
       </c>
     </row>
   </sheetData>
@@ -2974,7 +3139,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{256469AD-8C25-494B-B7FC-7D7B2DDE1DC0}">
-  <dimension ref="A1:C68"/>
+  <dimension ref="A1:C70"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="24" bestFit="1" customWidth="1"/>
@@ -3053,7 +3218,7 @@
         <v>22</v>
       </c>
       <c r="B7" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C7" t="s">
         <v>36</v>
@@ -3064,7 +3229,7 @@
         <v>22</v>
       </c>
       <c r="B8" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C8" t="s">
         <v>37</v>
@@ -3075,7 +3240,7 @@
         <v>24</v>
       </c>
       <c r="B9" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C9" t="s">
         <v>38</v>
@@ -3086,7 +3251,7 @@
         <v>24</v>
       </c>
       <c r="B10" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C10" t="s">
         <v>39</v>
@@ -3094,10 +3259,10 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B11" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C11" t="s">
         <v>42</v>
@@ -3105,10 +3270,10 @@
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B12" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C12" t="s">
         <v>43</v>
@@ -3116,10 +3281,10 @@
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B13" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C13" t="s">
         <v>44</v>
@@ -3127,79 +3292,79 @@
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B14" t="s">
+        <v>262</v>
+      </c>
+      <c r="C14" t="s">
         <v>263</v>
-      </c>
-      <c r="C14" t="s">
-        <v>264</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B15" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="C15" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B16" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="C16" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B17" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="C17" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B18" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="C18" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B19" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="C19" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B20" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="C20" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.2">
@@ -3232,7 +3397,7 @@
         <v>3</v>
       </c>
       <c r="C23" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.2">
@@ -3248,414 +3413,414 @@
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
+        <v>50</v>
+      </c>
+      <c r="B25">
+        <v>1</v>
+      </c>
+      <c r="C25" t="s">
         <v>51</v>
-      </c>
-      <c r="B25">
-        <v>1</v>
-      </c>
-      <c r="C25" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B26">
         <v>2</v>
       </c>
       <c r="C26" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B27">
         <v>1</v>
       </c>
       <c r="C27" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B28">
         <v>2</v>
       </c>
       <c r="C28" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B29">
         <v>3</v>
       </c>
       <c r="C29" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B30">
         <v>1</v>
       </c>
       <c r="C30" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B31">
         <v>2</v>
       </c>
       <c r="C31" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B32">
         <v>3</v>
       </c>
       <c r="C32" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B33">
         <v>4</v>
       </c>
       <c r="C33" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B34">
         <v>5</v>
       </c>
       <c r="C34" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B35">
         <v>6</v>
       </c>
       <c r="C35" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
+        <v>120</v>
+      </c>
+      <c r="B36">
+        <v>1</v>
+      </c>
+      <c r="C36" t="s">
         <v>121</v>
-      </c>
-      <c r="B36">
-        <v>1</v>
-      </c>
-      <c r="C36" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B37">
         <v>2</v>
       </c>
       <c r="C37" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B38">
         <v>3</v>
       </c>
       <c r="C38" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B39">
         <v>4</v>
       </c>
       <c r="C39" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
+        <v>127</v>
+      </c>
+      <c r="B40">
+        <v>1</v>
+      </c>
+      <c r="C40" t="s">
         <v>128</v>
-      </c>
-      <c r="B40">
-        <v>1</v>
-      </c>
-      <c r="C40" t="s">
-        <v>129</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B41">
         <v>2</v>
       </c>
       <c r="C41" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B42">
         <v>3</v>
       </c>
       <c r="C42" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B43">
         <v>4</v>
       </c>
       <c r="C43" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
+        <v>154</v>
+      </c>
+      <c r="B44">
+        <v>1</v>
+      </c>
+      <c r="C44" t="s">
         <v>155</v>
-      </c>
-      <c r="B44">
-        <v>1</v>
-      </c>
-      <c r="C44" t="s">
-        <v>156</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B45">
         <v>2</v>
       </c>
       <c r="C45" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B46">
         <v>3</v>
       </c>
       <c r="C46" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B47">
         <v>4</v>
       </c>
       <c r="C47" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B48">
         <v>1</v>
       </c>
       <c r="C48" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B49">
         <v>2</v>
       </c>
       <c r="C49" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B50">
         <v>3</v>
       </c>
       <c r="C50" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B51">
         <v>4</v>
       </c>
       <c r="C51" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B52">
         <v>1</v>
       </c>
       <c r="C52" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B53">
         <v>2</v>
       </c>
       <c r="C53" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B54">
         <v>3</v>
       </c>
       <c r="C54" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B55">
         <v>4</v>
       </c>
       <c r="C55" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B56">
         <v>5</v>
       </c>
       <c r="C56" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B57">
         <v>6</v>
       </c>
       <c r="C57" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B58">
         <v>7</v>
       </c>
       <c r="C58" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B59">
         <v>9999</v>
       </c>
       <c r="C59" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
+        <v>196</v>
+      </c>
+      <c r="B60">
+        <v>1</v>
+      </c>
+      <c r="C60" t="s">
         <v>197</v>
-      </c>
-      <c r="B60">
-        <v>1</v>
-      </c>
-      <c r="C60" t="s">
-        <v>198</v>
       </c>
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B61">
         <v>2</v>
       </c>
       <c r="C61" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B62">
         <v>3</v>
@@ -3666,40 +3831,40 @@
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="B63">
         <v>1</v>
       </c>
       <c r="C63" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="B64">
         <v>2</v>
       </c>
       <c r="C64" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="B65">
         <v>1</v>
       </c>
       <c r="C65" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
     </row>
     <row r="66" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="B66">
         <v>2</v>
@@ -3710,7 +3875,7 @@
     </row>
     <row r="67" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="B67">
         <v>3</v>
@@ -3721,13 +3886,35 @@
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="B68">
         <v>4</v>
       </c>
       <c r="C68" t="s">
         <v>48</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A69" t="s">
+        <v>289</v>
+      </c>
+      <c r="B69">
+        <v>1</v>
+      </c>
+      <c r="C69" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A70" t="s">
+        <v>289</v>
+      </c>
+      <c r="B70">
+        <v>2</v>
+      </c>
+      <c r="C70" t="s">
+        <v>291</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: industries, categories, subcategories
</commit_message>
<xml_diff>
--- a/backend/storage/schema/quotation_template.xlsx
+++ b/backend/storage/schema/quotation_template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/longlh123/Languages/GitHub/IPSOS-FINANCE-PAYMENT/backend/storage/schema/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88C394AF-70E7-3243-9774-52639ED80C15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F8F6FF6-8A0E-F640-ABDF-5B152D6CF046}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="6260" yWindow="3100" windowWidth="29040" windowHeight="17520" activeTab="1" xr2:uid="{C9138D76-07EC-41C4-8817-AFCBF30C50C2}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="575" uniqueCount="293">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="575" uniqueCount="295">
   <si>
     <t>field_name</t>
   </si>
@@ -520,9 +520,6 @@
     <t>dp_data_processing</t>
   </si>
   <si>
-    <t>Phương Pháp</t>
-  </si>
-  <si>
     <t>fieldwork_design</t>
   </si>
   <si>
@@ -538,33 +535,9 @@
     <t>excel:research_type</t>
   </si>
   <si>
-    <t>product_type</t>
-  </si>
-  <si>
     <t>Sản phẩm nghiên cứu</t>
   </si>
   <si>
-    <t>Nước giặt</t>
-  </si>
-  <si>
-    <t>Bột giặt</t>
-  </si>
-  <si>
-    <t>Nước rửa chén</t>
-  </si>
-  <si>
-    <t>Nước xả vải</t>
-  </si>
-  <si>
-    <t>Thuốc lá</t>
-  </si>
-  <si>
-    <t>Bia</t>
-  </si>
-  <si>
-    <t>excel:product_type</t>
-  </si>
-  <si>
     <t>Product Test - Monadic</t>
   </si>
   <si>
@@ -637,9 +610,6 @@
     <t>Tablet &lt; 9 inch</t>
   </si>
   <si>
-    <t>Không yêu cầu</t>
-  </si>
-  <si>
     <t>pm_required</t>
   </si>
   <si>
@@ -820,9 +790,6 @@
     <t>Paper</t>
   </si>
   <si>
-    <t>Nước ngọt</t>
-  </si>
-  <si>
     <t>placement</t>
   </si>
   <si>
@@ -917,6 +884,45 @@
   </si>
   <si>
     <t>travel_comment</t>
+  </si>
+  <si>
+    <t>Phương pháp nghiên cứu</t>
+  </si>
+  <si>
+    <t>product_classification</t>
+  </si>
+  <si>
+    <t>industry</t>
+  </si>
+  <si>
+    <t>category</t>
+  </si>
+  <si>
+    <t>subcategory</t>
+  </si>
+  <si>
+    <t>Ngành hàng</t>
+  </si>
+  <si>
+    <t>Nhóm sản phẩm</t>
+  </si>
+  <si>
+    <t>Loại sản phẩm</t>
+  </si>
+  <si>
+    <t>product_classification_config</t>
+  </si>
+  <si>
+    <t>db:industries</t>
+  </si>
+  <si>
+    <t>db:categories</t>
+  </si>
+  <si>
+    <t>db:subcategories</t>
+  </si>
+  <si>
+    <t>single-select</t>
   </si>
 </sst>
 </file>
@@ -1305,7 +1311,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6694FA44-4A7D-4629-A892-7DFDEEB80386}">
-  <dimension ref="A1:J25"/>
+  <dimension ref="A1:J26"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="24" bestFit="1" customWidth="1"/>
@@ -1483,7 +1489,7 @@
         <v>19</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>59</v>
+        <v>294</v>
       </c>
       <c r="D8">
         <v>1</v>
@@ -1534,10 +1540,10 @@
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B11" t="s">
-        <v>160</v>
+        <v>282</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>82</v>
@@ -1546,7 +1552,7 @@
         <v>1</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="H11">
         <v>12</v>
@@ -1554,19 +1560,19 @@
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>77</v>
+        <v>283</v>
       </c>
       <c r="B12" t="s">
-        <v>78</v>
+        <v>165</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>28</v>
+        <v>82</v>
       </c>
       <c r="D12">
         <v>1</v>
       </c>
       <c r="F12" t="s">
-        <v>79</v>
+        <v>290</v>
       </c>
       <c r="H12">
         <v>12</v>
@@ -1574,10 +1580,10 @@
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>61</v>
+        <v>77</v>
       </c>
       <c r="B13" t="s">
-        <v>60</v>
+        <v>78</v>
       </c>
       <c r="C13" s="1" t="s">
         <v>28</v>
@@ -1586,7 +1592,7 @@
         <v>1</v>
       </c>
       <c r="F13" t="s">
-        <v>62</v>
+        <v>79</v>
       </c>
       <c r="H13">
         <v>12</v>
@@ -1594,16 +1600,19 @@
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>278</v>
+        <v>61</v>
       </c>
       <c r="B14" t="s">
-        <v>279</v>
+        <v>60</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>82</v>
+        <v>28</v>
+      </c>
+      <c r="D14">
+        <v>1</v>
       </c>
       <c r="F14" t="s">
-        <v>280</v>
+        <v>62</v>
       </c>
       <c r="H14">
         <v>12</v>
@@ -1611,10 +1620,10 @@
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>231</v>
+        <v>267</v>
       </c>
       <c r="B15" t="s">
-        <v>232</v>
+        <v>268</v>
       </c>
       <c r="C15" s="1" t="s">
         <v>82</v>
@@ -1623,7 +1632,7 @@
         <v>1</v>
       </c>
       <c r="F15" t="s">
-        <v>231</v>
+        <v>269</v>
       </c>
       <c r="H15">
         <v>12</v>
@@ -1631,19 +1640,19 @@
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>111</v>
+        <v>221</v>
       </c>
       <c r="B16" t="s">
-        <v>110</v>
+        <v>222</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>28</v>
+        <v>82</v>
       </c>
       <c r="D16">
         <v>1</v>
       </c>
       <c r="F16" t="s">
-        <v>112</v>
+        <v>221</v>
       </c>
       <c r="H16">
         <v>12</v>
@@ -1651,19 +1660,19 @@
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="B17" t="s">
-        <v>116</v>
+        <v>110</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>82</v>
+        <v>28</v>
       </c>
       <c r="D17">
         <v>1</v>
       </c>
       <c r="F17" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
       <c r="H17">
         <v>12</v>
@@ -1671,10 +1680,10 @@
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>130</v>
+        <v>115</v>
       </c>
       <c r="B18" t="s">
-        <v>131</v>
+        <v>116</v>
       </c>
       <c r="C18" s="1" t="s">
         <v>82</v>
@@ -1683,7 +1692,7 @@
         <v>1</v>
       </c>
       <c r="F18" t="s">
-        <v>132</v>
+        <v>117</v>
       </c>
       <c r="H18">
         <v>12</v>
@@ -1691,10 +1700,10 @@
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>143</v>
+        <v>130</v>
       </c>
       <c r="B19" t="s">
-        <v>144</v>
+        <v>131</v>
       </c>
       <c r="C19" s="1" t="s">
         <v>82</v>
@@ -1703,7 +1712,7 @@
         <v>1</v>
       </c>
       <c r="F19" t="s">
-        <v>145</v>
+        <v>132</v>
       </c>
       <c r="H19">
         <v>12</v>
@@ -1711,16 +1720,19 @@
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>204</v>
+        <v>143</v>
       </c>
       <c r="B20" t="s">
-        <v>203</v>
+        <v>144</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>56</v>
+        <v>82</v>
       </c>
       <c r="D20">
         <v>1</v>
+      </c>
+      <c r="F20" t="s">
+        <v>145</v>
       </c>
       <c r="H20">
         <v>12</v>
@@ -1728,19 +1740,16 @@
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>200</v>
+        <v>194</v>
       </c>
       <c r="B21" t="s">
-        <v>201</v>
+        <v>193</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>23</v>
+        <v>56</v>
       </c>
       <c r="D21">
         <v>1</v>
-      </c>
-      <c r="G21" t="s">
-        <v>202</v>
       </c>
       <c r="H21">
         <v>12</v>
@@ -1748,19 +1757,19 @@
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>219</v>
+        <v>190</v>
       </c>
       <c r="B22" t="s">
-        <v>220</v>
+        <v>191</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>82</v>
+        <v>23</v>
       </c>
       <c r="D22">
         <v>1</v>
       </c>
-      <c r="F22" t="s">
-        <v>221</v>
+      <c r="G22" t="s">
+        <v>192</v>
       </c>
       <c r="H22">
         <v>12</v>
@@ -1768,19 +1777,19 @@
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
       <c r="B23" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>28</v>
+        <v>82</v>
       </c>
       <c r="D23">
         <v>1</v>
       </c>
       <c r="F23" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
       <c r="H23">
         <v>12</v>
@@ -1788,10 +1797,10 @@
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>211</v>
+        <v>195</v>
       </c>
       <c r="B24" t="s">
-        <v>212</v>
+        <v>203</v>
       </c>
       <c r="C24" s="1" t="s">
         <v>28</v>
@@ -1800,7 +1809,7 @@
         <v>1</v>
       </c>
       <c r="F24" t="s">
-        <v>214</v>
+        <v>196</v>
       </c>
       <c r="H24">
         <v>12</v>
@@ -1808,10 +1817,10 @@
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>283</v>
+        <v>201</v>
       </c>
       <c r="B25" t="s">
-        <v>284</v>
+        <v>202</v>
       </c>
       <c r="C25" s="1" t="s">
         <v>28</v>
@@ -1820,9 +1829,29 @@
         <v>1</v>
       </c>
       <c r="F25" t="s">
-        <v>285</v>
+        <v>204</v>
       </c>
       <c r="H25">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A26" t="s">
+        <v>272</v>
+      </c>
+      <c r="B26" t="s">
+        <v>273</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="D26">
+        <v>1</v>
+      </c>
+      <c r="F26" t="s">
+        <v>274</v>
+      </c>
+      <c r="H26">
         <v>12</v>
       </c>
     </row>
@@ -1834,13 +1863,13 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F2B8FC54-75D4-4AC2-B92C-338AB72929A6}">
-  <dimension ref="A1:H59"/>
+  <dimension ref="A1:H61"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="29.83203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="36" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="31.5" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.83203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.33203125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="12.6640625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="25" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="11" bestFit="1" customWidth="1"/>
@@ -1874,7 +1903,7 @@
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B2" t="s">
         <v>75</v>
@@ -1893,18 +1922,18 @@
         <v>67</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B3" t="s">
-        <v>193</v>
+        <v>184</v>
       </c>
       <c r="C3" t="s">
-        <v>194</v>
+        <v>185</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>59</v>
@@ -1914,21 +1943,21 @@
       </c>
       <c r="F3" s="1"/>
       <c r="G3" t="s">
-        <v>195</v>
+        <v>186</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="B4" t="s">
+        <v>163</v>
+      </c>
+      <c r="C4" t="s">
         <v>162</v>
-      </c>
-      <c r="B4" t="s">
-        <v>164</v>
-      </c>
-      <c r="C4" t="s">
-        <v>163</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>59</v>
@@ -1938,21 +1967,21 @@
       </c>
       <c r="F4" s="1"/>
       <c r="G4" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>191</v>
+        <v>182</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B5" t="s">
-        <v>166</v>
+        <v>45</v>
       </c>
       <c r="C5" t="s">
-        <v>167</v>
+        <v>20</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>59</v>
@@ -1962,98 +1991,103 @@
       </c>
       <c r="F5" s="1"/>
       <c r="G5" t="s">
-        <v>174</v>
+        <v>76</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B6" t="s">
-        <v>45</v>
+        <v>178</v>
       </c>
       <c r="C6" t="s">
-        <v>20</v>
+        <v>179</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="E6">
         <v>1</v>
       </c>
       <c r="F6" s="1"/>
-      <c r="G6" t="s">
-        <v>76</v>
-      </c>
       <c r="H6" s="1" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A7" s="2" t="s">
-        <v>162</v>
+      <c r="A7" t="s">
+        <v>290</v>
       </c>
       <c r="B7" t="s">
-        <v>187</v>
+        <v>284</v>
       </c>
       <c r="C7" t="s">
-        <v>188</v>
+        <v>287</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>56</v>
+        <v>294</v>
       </c>
       <c r="E7">
         <v>1</v>
       </c>
       <c r="F7" s="1"/>
+      <c r="G7" t="s">
+        <v>291</v>
+      </c>
       <c r="H7" s="1" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>79</v>
+        <v>290</v>
       </c>
       <c r="B8" t="s">
-        <v>80</v>
+        <v>285</v>
       </c>
       <c r="C8" t="s">
-        <v>41</v>
+        <v>288</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>59</v>
+        <v>294</v>
       </c>
       <c r="E8">
         <v>1</v>
       </c>
+      <c r="F8" s="1"/>
       <c r="G8" t="s">
-        <v>81</v>
+        <v>292</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>79</v>
+        <v>290</v>
       </c>
       <c r="B9" t="s">
-        <v>25</v>
+        <v>286</v>
       </c>
       <c r="C9" t="s">
-        <v>104</v>
+        <v>289</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>27</v>
+        <v>59</v>
       </c>
       <c r="E9">
         <v>1</v>
       </c>
+      <c r="F9" s="1"/>
+      <c r="G9" t="s">
+        <v>293</v>
+      </c>
       <c r="H9" s="1" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.2">
@@ -2061,62 +2095,62 @@
         <v>79</v>
       </c>
       <c r="B10" t="s">
-        <v>26</v>
+        <v>80</v>
       </c>
       <c r="C10" t="s">
-        <v>105</v>
+        <v>41</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>27</v>
+        <v>294</v>
       </c>
       <c r="E10">
         <v>1</v>
       </c>
+      <c r="G10" t="s">
+        <v>81</v>
+      </c>
       <c r="H10" s="1" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>62</v>
+        <v>79</v>
       </c>
       <c r="B11" t="s">
-        <v>281</v>
+        <v>25</v>
       </c>
       <c r="C11" t="s">
-        <v>282</v>
+        <v>104</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>6</v>
+        <v>27</v>
       </c>
       <c r="E11">
         <v>1</v>
       </c>
       <c r="H11" s="1" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>62</v>
+        <v>79</v>
       </c>
       <c r="B12" t="s">
-        <v>83</v>
+        <v>26</v>
       </c>
       <c r="C12" t="s">
-        <v>84</v>
+        <v>105</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="E12">
         <v>1</v>
       </c>
-      <c r="G12" t="s">
-        <v>85</v>
-      </c>
       <c r="H12" s="1" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
@@ -2124,10 +2158,10 @@
         <v>62</v>
       </c>
       <c r="B13" t="s">
-        <v>89</v>
+        <v>270</v>
       </c>
       <c r="C13" t="s">
-        <v>90</v>
+        <v>271</v>
       </c>
       <c r="D13" s="1" t="s">
         <v>6</v>
@@ -2136,81 +2170,84 @@
         <v>1</v>
       </c>
       <c r="H13" s="1" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>280</v>
+        <v>62</v>
       </c>
       <c r="B14" t="s">
-        <v>91</v>
+        <v>83</v>
       </c>
       <c r="C14" t="s">
-        <v>92</v>
+        <v>84</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>59</v>
+        <v>294</v>
       </c>
       <c r="E14">
         <v>1</v>
       </c>
       <c r="G14" t="s">
-        <v>93</v>
+        <v>85</v>
       </c>
       <c r="H14" s="1" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>280</v>
+        <v>62</v>
       </c>
       <c r="B15" t="s">
-        <v>102</v>
+        <v>89</v>
       </c>
       <c r="C15" t="s">
-        <v>103</v>
+        <v>90</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>56</v>
+        <v>6</v>
       </c>
       <c r="E15">
         <v>1</v>
       </c>
       <c r="H15" s="1" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>280</v>
+        <v>269</v>
       </c>
       <c r="B16" t="s">
-        <v>100</v>
+        <v>91</v>
       </c>
       <c r="C16" t="s">
-        <v>101</v>
+        <v>92</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="E16">
         <v>1</v>
       </c>
+      <c r="G16" t="s">
+        <v>93</v>
+      </c>
       <c r="H16" s="1" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>280</v>
+        <v>269</v>
       </c>
       <c r="B17" t="s">
-        <v>247</v>
+        <v>102</v>
       </c>
       <c r="C17" t="s">
-        <v>275</v>
+        <v>103</v>
       </c>
       <c r="D17" s="1" t="s">
         <v>56</v>
@@ -2219,18 +2256,18 @@
         <v>1</v>
       </c>
       <c r="H17" s="1" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>280</v>
+        <v>269</v>
       </c>
       <c r="B18" t="s">
-        <v>107</v>
+        <v>100</v>
       </c>
       <c r="C18" t="s">
-        <v>108</v>
+        <v>101</v>
       </c>
       <c r="D18" s="1" t="s">
         <v>56</v>
@@ -2239,60 +2276,58 @@
         <v>1</v>
       </c>
       <c r="H18" s="1" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>231</v>
+        <v>269</v>
       </c>
       <c r="B19" t="s">
-        <v>179</v>
+        <v>237</v>
       </c>
       <c r="C19" t="s">
-        <v>182</v>
+        <v>264</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>27</v>
+        <v>56</v>
       </c>
       <c r="E19">
         <v>1</v>
       </c>
-      <c r="F19" s="1"/>
       <c r="H19" s="1" t="s">
-        <v>191</v>
+        <v>183</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>231</v>
+        <v>269</v>
       </c>
       <c r="B20" t="s">
-        <v>180</v>
+        <v>107</v>
       </c>
       <c r="C20" t="s">
-        <v>181</v>
+        <v>108</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>27</v>
+        <v>56</v>
       </c>
       <c r="E20">
         <v>1</v>
       </c>
-      <c r="F20" s="1"/>
       <c r="H20" s="1" t="s">
-        <v>191</v>
+        <v>183</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>231</v>
+        <v>221</v>
       </c>
       <c r="B21" t="s">
-        <v>183</v>
+        <v>170</v>
       </c>
       <c r="C21" t="s">
-        <v>185</v>
+        <v>173</v>
       </c>
       <c r="D21" s="1" t="s">
         <v>27</v>
@@ -2302,18 +2337,18 @@
       </c>
       <c r="F21" s="1"/>
       <c r="H21" s="1" t="s">
-        <v>191</v>
+        <v>182</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>231</v>
+        <v>221</v>
       </c>
       <c r="B22" t="s">
-        <v>184</v>
+        <v>171</v>
       </c>
       <c r="C22" t="s">
-        <v>186</v>
+        <v>172</v>
       </c>
       <c r="D22" s="1" t="s">
         <v>27</v>
@@ -2323,18 +2358,18 @@
       </c>
       <c r="F22" s="1"/>
       <c r="H22" s="1" t="s">
-        <v>191</v>
+        <v>182</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>231</v>
+        <v>221</v>
       </c>
       <c r="B23" t="s">
-        <v>189</v>
+        <v>174</v>
       </c>
       <c r="C23" t="s">
-        <v>190</v>
+        <v>176</v>
       </c>
       <c r="D23" s="1" t="s">
         <v>27</v>
@@ -2344,177 +2379,174 @@
       </c>
       <c r="F23" s="1"/>
       <c r="H23" s="1" t="s">
-        <v>191</v>
+        <v>182</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>231</v>
+        <v>221</v>
       </c>
       <c r="B24" t="s">
-        <v>233</v>
+        <v>175</v>
       </c>
       <c r="C24" t="s">
-        <v>234</v>
+        <v>177</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>56</v>
+        <v>27</v>
       </c>
       <c r="E24">
         <v>1</v>
       </c>
       <c r="F24" s="1"/>
       <c r="H24" s="1" t="s">
-        <v>191</v>
+        <v>182</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>231</v>
+        <v>221</v>
       </c>
       <c r="B25" t="s">
-        <v>254</v>
+        <v>180</v>
       </c>
       <c r="C25" t="s">
-        <v>255</v>
+        <v>181</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="E25">
         <v>1</v>
       </c>
       <c r="F25" s="1"/>
-      <c r="G25" t="s">
-        <v>50</v>
-      </c>
       <c r="H25" s="1" t="s">
-        <v>191</v>
+        <v>182</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>231</v>
+        <v>221</v>
       </c>
       <c r="B26" t="s">
-        <v>256</v>
+        <v>223</v>
       </c>
       <c r="C26" t="s">
-        <v>257</v>
+        <v>224</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>23</v>
+        <v>56</v>
       </c>
       <c r="E26">
         <v>1</v>
       </c>
       <c r="F26" s="1"/>
-      <c r="G26" t="s">
-        <v>258</v>
-      </c>
       <c r="H26" s="1" t="s">
-        <v>191</v>
+        <v>182</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>231</v>
+        <v>221</v>
       </c>
       <c r="B27" t="s">
-        <v>235</v>
+        <v>244</v>
       </c>
       <c r="C27" t="s">
-        <v>240</v>
+        <v>245</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>59</v>
+        <v>23</v>
       </c>
       <c r="E27">
         <v>1</v>
       </c>
       <c r="F27" s="1"/>
       <c r="G27" t="s">
-        <v>236</v>
+        <v>50</v>
       </c>
       <c r="H27" s="1" t="s">
-        <v>191</v>
+        <v>182</v>
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>231</v>
+        <v>221</v>
       </c>
       <c r="B28" t="s">
-        <v>239</v>
+        <v>246</v>
       </c>
       <c r="C28" t="s">
-        <v>241</v>
+        <v>247</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>56</v>
+        <v>23</v>
       </c>
       <c r="E28">
         <v>1</v>
       </c>
       <c r="F28" s="1"/>
+      <c r="G28" t="s">
+        <v>248</v>
+      </c>
       <c r="H28" s="1" t="s">
-        <v>191</v>
+        <v>182</v>
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>231</v>
+        <v>221</v>
       </c>
       <c r="B29" t="s">
-        <v>242</v>
+        <v>225</v>
       </c>
       <c r="C29" t="s">
-        <v>243</v>
+        <v>230</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="E29">
         <v>1</v>
       </c>
       <c r="F29" s="1"/>
+      <c r="G29" t="s">
+        <v>226</v>
+      </c>
       <c r="H29" s="1" t="s">
-        <v>191</v>
+        <v>182</v>
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
+        <v>221</v>
+      </c>
+      <c r="B30" t="s">
+        <v>229</v>
+      </c>
+      <c r="C30" t="s">
         <v>231</v>
       </c>
-      <c r="B30" t="s">
-        <v>253</v>
-      </c>
-      <c r="C30" t="s">
-        <v>245</v>
-      </c>
       <c r="D30" s="1" t="s">
-        <v>23</v>
+        <v>56</v>
       </c>
       <c r="E30">
         <v>1</v>
       </c>
       <c r="F30" s="1"/>
-      <c r="G30" t="s">
-        <v>50</v>
-      </c>
       <c r="H30" s="1" t="s">
-        <v>191</v>
+        <v>182</v>
       </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>231</v>
+        <v>221</v>
       </c>
       <c r="B31" t="s">
-        <v>246</v>
+        <v>232</v>
       </c>
       <c r="C31" t="s">
-        <v>244</v>
+        <v>233</v>
       </c>
       <c r="D31" s="1" t="s">
         <v>56</v>
@@ -2524,122 +2556,121 @@
       </c>
       <c r="F31" s="1"/>
       <c r="H31" s="1" t="s">
-        <v>191</v>
+        <v>182</v>
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>231</v>
+        <v>221</v>
       </c>
       <c r="B32" t="s">
-        <v>247</v>
+        <v>243</v>
       </c>
       <c r="C32" t="s">
-        <v>248</v>
+        <v>235</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>56</v>
+        <v>23</v>
       </c>
       <c r="E32">
         <v>1</v>
       </c>
       <c r="F32" s="1"/>
+      <c r="G32" t="s">
+        <v>50</v>
+      </c>
       <c r="H32" s="1" t="s">
-        <v>191</v>
+        <v>182</v>
       </c>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>231</v>
+        <v>221</v>
       </c>
       <c r="B33" t="s">
-        <v>249</v>
+        <v>236</v>
       </c>
       <c r="C33" t="s">
-        <v>251</v>
+        <v>234</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>23</v>
+        <v>56</v>
       </c>
       <c r="E33">
         <v>1</v>
       </c>
       <c r="F33" s="1"/>
-      <c r="G33" t="s">
-        <v>50</v>
-      </c>
       <c r="H33" s="1" t="s">
-        <v>191</v>
+        <v>182</v>
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>231</v>
+        <v>221</v>
       </c>
       <c r="B34" t="s">
-        <v>250</v>
+        <v>237</v>
       </c>
       <c r="C34" t="s">
-        <v>252</v>
+        <v>238</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>23</v>
+        <v>56</v>
       </c>
       <c r="E34">
         <v>1</v>
       </c>
       <c r="F34" s="1"/>
-      <c r="G34" t="s">
-        <v>50</v>
-      </c>
       <c r="H34" s="1" t="s">
-        <v>191</v>
+        <v>182</v>
       </c>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>112</v>
+        <v>221</v>
       </c>
       <c r="B35" t="s">
-        <v>109</v>
+        <v>239</v>
       </c>
       <c r="C35" t="s">
-        <v>114</v>
+        <v>241</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>59</v>
+        <v>23</v>
       </c>
       <c r="E35">
         <v>1</v>
       </c>
+      <c r="F35" s="1"/>
       <c r="G35" t="s">
-        <v>113</v>
+        <v>50</v>
       </c>
       <c r="H35" s="1" t="s">
-        <v>192</v>
+        <v>182</v>
       </c>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>112</v>
+        <v>221</v>
       </c>
       <c r="B36" t="s">
-        <v>226</v>
+        <v>240</v>
       </c>
       <c r="C36" t="s">
-        <v>228</v>
+        <v>242</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="E36">
         <v>1</v>
       </c>
-      <c r="F36">
-        <v>0</v>
+      <c r="F36" s="1"/>
+      <c r="G36" t="s">
+        <v>50</v>
       </c>
       <c r="H36" s="1" t="s">
-        <v>192</v>
+        <v>182</v>
       </c>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.2">
@@ -2647,68 +2678,68 @@
         <v>112</v>
       </c>
       <c r="B37" t="s">
-        <v>227</v>
+        <v>109</v>
       </c>
       <c r="C37" t="s">
-        <v>229</v>
+        <v>114</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>27</v>
+        <v>294</v>
       </c>
       <c r="E37">
-        <v>0</v>
-      </c>
-      <c r="F37">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="G37" t="s">
+        <v>113</v>
       </c>
       <c r="H37" s="1" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
       <c r="B38" t="s">
-        <v>134</v>
+        <v>216</v>
       </c>
       <c r="C38" t="s">
-        <v>118</v>
+        <v>218</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>59</v>
+        <v>27</v>
       </c>
       <c r="E38">
         <v>1</v>
       </c>
-      <c r="G38" t="s">
-        <v>119</v>
+      <c r="F38">
+        <v>0</v>
       </c>
       <c r="H38" s="1" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
       <c r="B39" t="s">
-        <v>135</v>
+        <v>217</v>
       </c>
       <c r="C39" t="s">
-        <v>125</v>
+        <v>219</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>59</v>
+        <v>27</v>
       </c>
       <c r="E39">
-        <v>1</v>
-      </c>
-      <c r="G39" t="s">
-        <v>126</v>
+        <v>0</v>
+      </c>
+      <c r="F39">
+        <v>0</v>
       </c>
       <c r="H39" s="1" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.2">
@@ -2716,59 +2747,65 @@
         <v>117</v>
       </c>
       <c r="B40" t="s">
-        <v>276</v>
+        <v>134</v>
       </c>
       <c r="C40" t="s">
-        <v>277</v>
+        <v>118</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>56</v>
+        <v>294</v>
       </c>
       <c r="E40">
         <v>1</v>
       </c>
+      <c r="G40" t="s">
+        <v>119</v>
+      </c>
       <c r="H40" s="1" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>132</v>
+        <v>117</v>
       </c>
       <c r="B41" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
       <c r="C41" t="s">
-        <v>133</v>
+        <v>125</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="E41">
         <v>1</v>
       </c>
+      <c r="G41" t="s">
+        <v>126</v>
+      </c>
       <c r="H41" s="1" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>132</v>
+        <v>117</v>
       </c>
       <c r="B42" t="s">
-        <v>136</v>
+        <v>265</v>
       </c>
       <c r="C42" t="s">
-        <v>137</v>
+        <v>266</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>27</v>
+        <v>56</v>
       </c>
       <c r="E42">
         <v>1</v>
       </c>
       <c r="H42" s="1" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.2">
@@ -2776,10 +2813,10 @@
         <v>132</v>
       </c>
       <c r="B43" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C43" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="D43" s="1" t="s">
         <v>56</v>
@@ -2788,7 +2825,7 @@
         <v>1</v>
       </c>
       <c r="H43" s="1" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.2">
@@ -2796,65 +2833,59 @@
         <v>132</v>
       </c>
       <c r="B44" t="s">
-        <v>142</v>
+        <v>136</v>
       </c>
       <c r="C44" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>56</v>
+        <v>27</v>
       </c>
       <c r="E44">
         <v>1</v>
       </c>
       <c r="H44" s="1" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>145</v>
+        <v>132</v>
       </c>
       <c r="B45" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
       <c r="C45" t="s">
-        <v>148</v>
+        <v>138</v>
       </c>
       <c r="D45" s="1" t="s">
-        <v>23</v>
+        <v>56</v>
       </c>
       <c r="E45">
         <v>1</v>
       </c>
-      <c r="G45" t="s">
-        <v>50</v>
-      </c>
       <c r="H45" s="1" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>145</v>
+        <v>132</v>
       </c>
       <c r="B46" t="s">
-        <v>147</v>
+        <v>142</v>
       </c>
       <c r="C46" t="s">
-        <v>149</v>
+        <v>139</v>
       </c>
       <c r="D46" s="1" t="s">
-        <v>23</v>
+        <v>56</v>
       </c>
       <c r="E46">
         <v>1</v>
       </c>
-      <c r="G46" t="s">
-        <v>50</v>
-      </c>
       <c r="H46" s="1" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.2">
@@ -2862,22 +2893,22 @@
         <v>145</v>
       </c>
       <c r="B47" t="s">
-        <v>159</v>
+        <v>146</v>
       </c>
       <c r="C47" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="D47" s="1" t="s">
-        <v>59</v>
+        <v>23</v>
       </c>
       <c r="E47">
         <v>1</v>
       </c>
       <c r="G47" t="s">
-        <v>153</v>
+        <v>50</v>
       </c>
       <c r="H47" s="1" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.2">
@@ -2885,50 +2916,56 @@
         <v>145</v>
       </c>
       <c r="B48" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="C48" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="D48" s="1" t="s">
-        <v>56</v>
+        <v>23</v>
       </c>
       <c r="E48">
         <v>1</v>
       </c>
+      <c r="G48" t="s">
+        <v>50</v>
+      </c>
       <c r="H48" s="1" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
-        <v>221</v>
+        <v>145</v>
       </c>
       <c r="B49" t="s">
-        <v>222</v>
+        <v>159</v>
       </c>
       <c r="C49" t="s">
-        <v>223</v>
+        <v>150</v>
       </c>
       <c r="D49" s="1" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="E49">
         <v>1</v>
       </c>
+      <c r="G49" t="s">
+        <v>153</v>
+      </c>
       <c r="H49" s="1" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
     </row>
     <row r="50" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
-        <v>221</v>
+        <v>145</v>
       </c>
       <c r="B50" t="s">
-        <v>224</v>
+        <v>151</v>
       </c>
       <c r="C50" t="s">
-        <v>225</v>
+        <v>152</v>
       </c>
       <c r="D50" s="1" t="s">
         <v>56</v>
@@ -2937,209 +2974,250 @@
         <v>1</v>
       </c>
       <c r="H50" s="1" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
       <c r="B51" t="s">
-        <v>208</v>
+        <v>212</v>
       </c>
       <c r="C51" t="s">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="D51" s="1" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="E51">
         <v>1</v>
       </c>
-      <c r="G51" t="s">
-        <v>113</v>
-      </c>
       <c r="H51" s="1" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
     </row>
     <row r="52" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
       <c r="B52" t="s">
-        <v>207</v>
+        <v>214</v>
       </c>
       <c r="C52" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="D52" s="1" t="s">
-        <v>27</v>
+        <v>56</v>
       </c>
       <c r="E52">
         <v>1</v>
       </c>
       <c r="H52" s="1" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
     </row>
     <row r="53" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
-        <v>206</v>
+        <v>196</v>
       </c>
       <c r="B53" t="s">
-        <v>210</v>
+        <v>198</v>
       </c>
       <c r="C53" t="s">
-        <v>188</v>
+        <v>199</v>
       </c>
       <c r="D53" s="1" t="s">
-        <v>6</v>
+        <v>294</v>
       </c>
       <c r="E53">
         <v>1</v>
       </c>
+      <c r="G53" t="s">
+        <v>113</v>
+      </c>
       <c r="H53" s="1" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
     </row>
     <row r="54" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
-        <v>214</v>
+        <v>196</v>
       </c>
       <c r="B54" t="s">
-        <v>216</v>
+        <v>197</v>
       </c>
       <c r="C54" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="D54" s="1" t="s">
-        <v>59</v>
+        <v>27</v>
       </c>
       <c r="E54">
         <v>1</v>
       </c>
-      <c r="G54" t="s">
-        <v>113</v>
-      </c>
       <c r="H54" s="1" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
     </row>
     <row r="55" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
-        <v>214</v>
+        <v>196</v>
       </c>
       <c r="B55" t="s">
-        <v>215</v>
+        <v>200</v>
       </c>
       <c r="C55" t="s">
-        <v>218</v>
+        <v>179</v>
       </c>
       <c r="D55" s="1" t="s">
-        <v>27</v>
+        <v>6</v>
       </c>
       <c r="E55">
         <v>1</v>
       </c>
       <c r="H55" s="1" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
     </row>
     <row r="56" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
-        <v>214</v>
+        <v>204</v>
       </c>
       <c r="B56" t="s">
-        <v>217</v>
+        <v>206</v>
       </c>
       <c r="C56" t="s">
-        <v>188</v>
+        <v>199</v>
       </c>
       <c r="D56" s="1" t="s">
-        <v>6</v>
+        <v>294</v>
       </c>
       <c r="E56">
         <v>1</v>
       </c>
+      <c r="G56" t="s">
+        <v>113</v>
+      </c>
       <c r="H56" s="1" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
     </row>
     <row r="57" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
-        <v>285</v>
+        <v>204</v>
       </c>
       <c r="B57" t="s">
-        <v>109</v>
+        <v>205</v>
       </c>
       <c r="C57" t="s">
-        <v>114</v>
+        <v>208</v>
       </c>
       <c r="D57" s="1" t="s">
-        <v>59</v>
+        <v>27</v>
       </c>
       <c r="E57">
         <v>1</v>
       </c>
-      <c r="G57" t="s">
-        <v>113</v>
-      </c>
       <c r="H57" s="1" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
-        <v>285</v>
+        <v>204</v>
       </c>
       <c r="B58" t="s">
-        <v>286</v>
+        <v>207</v>
       </c>
       <c r="C58" t="s">
-        <v>287</v>
+        <v>179</v>
       </c>
       <c r="D58" s="1" t="s">
-        <v>59</v>
+        <v>6</v>
       </c>
       <c r="E58">
         <v>1</v>
       </c>
-      <c r="G58" t="s">
-        <v>288</v>
-      </c>
       <c r="H58" s="1" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
     </row>
     <row r="59" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
-        <v>285</v>
+        <v>274</v>
       </c>
       <c r="B59" t="s">
-        <v>292</v>
+        <v>109</v>
       </c>
       <c r="C59" t="s">
-        <v>188</v>
+        <v>114</v>
       </c>
       <c r="D59" s="1" t="s">
+        <v>294</v>
+      </c>
+      <c r="E59">
+        <v>1</v>
+      </c>
+      <c r="G59" t="s">
+        <v>113</v>
+      </c>
+      <c r="H59" s="1" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="60" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A60" t="s">
+        <v>274</v>
+      </c>
+      <c r="B60" t="s">
+        <v>275</v>
+      </c>
+      <c r="C60" t="s">
+        <v>276</v>
+      </c>
+      <c r="D60" s="1" t="s">
+        <v>294</v>
+      </c>
+      <c r="E60">
+        <v>1</v>
+      </c>
+      <c r="G60" t="s">
+        <v>277</v>
+      </c>
+      <c r="H60" s="1" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="61" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A61" t="s">
+        <v>274</v>
+      </c>
+      <c r="B61" t="s">
+        <v>281</v>
+      </c>
+      <c r="C61" t="s">
+        <v>179</v>
+      </c>
+      <c r="D61" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="E59">
-        <v>1</v>
-      </c>
-      <c r="H59" s="1" t="s">
-        <v>192</v>
+      <c r="E61">
+        <v>1</v>
+      </c>
+      <c r="H61" s="1" t="s">
+        <v>183</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{256469AD-8C25-494B-B7FC-7D7B2DDE1DC0}">
-  <dimension ref="A1:C70"/>
+  <dimension ref="A1:C62"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="24" bestFit="1" customWidth="1"/>
@@ -3295,10 +3373,10 @@
         <v>80</v>
       </c>
       <c r="B14" t="s">
-        <v>262</v>
+        <v>251</v>
       </c>
       <c r="C14" t="s">
-        <v>263</v>
+        <v>252</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.2">
@@ -3306,10 +3384,10 @@
         <v>80</v>
       </c>
       <c r="B15" t="s">
-        <v>261</v>
+        <v>250</v>
       </c>
       <c r="C15" t="s">
-        <v>264</v>
+        <v>253</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.2">
@@ -3317,10 +3395,10 @@
         <v>80</v>
       </c>
       <c r="B16" t="s">
-        <v>265</v>
+        <v>254</v>
       </c>
       <c r="C16" t="s">
-        <v>270</v>
+        <v>259</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.2">
@@ -3328,10 +3406,10 @@
         <v>80</v>
       </c>
       <c r="B17" t="s">
-        <v>266</v>
+        <v>255</v>
       </c>
       <c r="C17" t="s">
-        <v>271</v>
+        <v>260</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.2">
@@ -3339,10 +3417,10 @@
         <v>80</v>
       </c>
       <c r="B18" t="s">
-        <v>267</v>
+        <v>256</v>
       </c>
       <c r="C18" t="s">
-        <v>272</v>
+        <v>261</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.2">
@@ -3350,10 +3428,10 @@
         <v>80</v>
       </c>
       <c r="B19" t="s">
-        <v>268</v>
+        <v>257</v>
       </c>
       <c r="C19" t="s">
-        <v>273</v>
+        <v>262</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.2">
@@ -3361,10 +3439,10 @@
         <v>80</v>
       </c>
       <c r="B20" t="s">
-        <v>269</v>
+        <v>258</v>
       </c>
       <c r="C20" t="s">
-        <v>274</v>
+        <v>263</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.2">
@@ -3397,7 +3475,7 @@
         <v>3</v>
       </c>
       <c r="C23" t="s">
-        <v>230</v>
+        <v>220</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.2">
@@ -3666,255 +3744,167 @@
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B48">
         <v>1</v>
       </c>
       <c r="C48" t="s">
-        <v>175</v>
+        <v>166</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B49">
         <v>2</v>
       </c>
       <c r="C49" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B50">
         <v>3</v>
       </c>
       <c r="C50" t="s">
-        <v>176</v>
+        <v>167</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B51">
         <v>4</v>
       </c>
       <c r="C51" t="s">
-        <v>178</v>
+        <v>169</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
-        <v>166</v>
+        <v>187</v>
       </c>
       <c r="B52">
         <v>1</v>
       </c>
       <c r="C52" t="s">
-        <v>168</v>
+        <v>188</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
-        <v>166</v>
+        <v>187</v>
       </c>
       <c r="B53">
         <v>2</v>
       </c>
       <c r="C53" t="s">
-        <v>169</v>
+        <v>189</v>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
-        <v>166</v>
+        <v>187</v>
       </c>
       <c r="B54">
         <v>3</v>
       </c>
       <c r="C54" t="s">
-        <v>170</v>
+        <v>39</v>
       </c>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
-        <v>166</v>
+        <v>225</v>
       </c>
       <c r="B55">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C55" t="s">
-        <v>171</v>
+        <v>227</v>
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
-        <v>166</v>
+        <v>225</v>
       </c>
       <c r="B56">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="C56" t="s">
-        <v>172</v>
+        <v>228</v>
       </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
-        <v>166</v>
+        <v>246</v>
       </c>
       <c r="B57">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="C57" t="s">
-        <v>173</v>
+        <v>249</v>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
-        <v>166</v>
+        <v>246</v>
       </c>
       <c r="B58">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="C58" t="s">
-        <v>260</v>
+        <v>37</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
-        <v>166</v>
+        <v>246</v>
       </c>
       <c r="B59">
-        <v>9999</v>
+        <v>3</v>
       </c>
       <c r="C59" t="s">
-        <v>199</v>
+        <v>36</v>
       </c>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
-        <v>196</v>
+        <v>246</v>
       </c>
       <c r="B60">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C60" t="s">
-        <v>197</v>
+        <v>48</v>
       </c>
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
-        <v>196</v>
+        <v>278</v>
       </c>
       <c r="B61">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C61" t="s">
-        <v>198</v>
+        <v>279</v>
       </c>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
-        <v>196</v>
+        <v>278</v>
       </c>
       <c r="B62">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C62" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A63" t="s">
-        <v>235</v>
-      </c>
-      <c r="B63">
-        <v>1</v>
-      </c>
-      <c r="C63" t="s">
-        <v>237</v>
-      </c>
-    </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A64" t="s">
-        <v>235</v>
-      </c>
-      <c r="B64">
-        <v>2</v>
-      </c>
-      <c r="C64" t="s">
-        <v>238</v>
-      </c>
-    </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A65" t="s">
-        <v>256</v>
-      </c>
-      <c r="B65">
-        <v>1</v>
-      </c>
-      <c r="C65" t="s">
-        <v>259</v>
-      </c>
-    </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A66" t="s">
-        <v>256</v>
-      </c>
-      <c r="B66">
-        <v>2</v>
-      </c>
-      <c r="C66" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A67" t="s">
-        <v>256</v>
-      </c>
-      <c r="B67">
-        <v>3</v>
-      </c>
-      <c r="C67" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A68" t="s">
-        <v>256</v>
-      </c>
-      <c r="B68">
-        <v>4</v>
-      </c>
-      <c r="C68" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A69" t="s">
-        <v>289</v>
-      </c>
-      <c r="B69">
-        <v>1</v>
-      </c>
-      <c r="C69" t="s">
-        <v>290</v>
-      </c>
-    </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A70" t="s">
-        <v>289</v>
-      </c>
-      <c r="B70">
-        <v>2</v>
-      </c>
-      <c r="C70" t="s">
-        <v>291</v>
+        <v>280</v>
       </c>
     </row>
   </sheetData>

</xml_diff>